<commit_message>
Checkpoint: 18 file(s) across testrail-import, build/report-suite/viu-2026-08-03, build/report-suite/cases, build/report-suite/verifier-fixes-2026-08-03
Unattended checkpoint sweep 19 (concurrent multi-worker session).
Additive commit of hash-stable, secret-scanned paths only.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AZ5XzKsK9wv7M41cSPaMyg
</commit_message>
<xml_diff>
--- a/testrail-import/Report-Suite_Sales-By-Customer-Report_testrail-import.xlsx
+++ b/testrail-import/Report-Suite_Sales-By-Customer-Report_testrail-import.xlsx
@@ -828,7 +828,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>SV-8601 (SBC spec v12 2026-07-29 Story 2 S2-R1; S2-R2 — S2-R2 CLOSES the eleven-option list and its order itself; so the closed list IS the requirement; re-check this case whenever S2-R2 changes)</t>
+          <t>SV-8601 (SBC spec v13 2026-07-31 Story 2 S2-R1; S2-R2 — S2-R2 CLOSES the eleven-option list and its order itself; so the closed list IS the requirement; re-check this case whenever S2-R2 changes)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
@@ -975,7 +975,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>SV-8602 (SBC spec v12 2026-07-29 Story 3 S3-R1; S3-R2; S3-R3; S3-R4; S3-R5; S3-R6 — S3-R2 CLOSES the list itself ("exactly three options ... in this order"); so the closed list IS the requirement)</t>
+          <t>SV-8602 (SBC spec v13 2026-07-31 Story 3 S3-R1; S3-R2; S3-R3; S3-R4; S3-R5; S3-R6 — S3-R2 CLOSES the list itself ("exactly three options ... in this order"); so the closed list IS the requirement)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr"/>
@@ -2583,7 +2583,7 @@
       </c>
       <c r="H44" s="2" t="inlineStr">
         <is>
-          <t>SV-8605 (SBC spec v12 2026-07-29 §2; §4 Terminology; Story 7 S7-R6; Story 11 S11-R1 — §2/S7-R6 CLOSE the financial-column list and its order; Location is an identifier column not a financial one [S4-R12; S20-R19] so it never enters this list)</t>
+          <t>SV-8605 (SBC spec v13 2026-07-31 §2; §4 Terminology; Story 7 S7-R6; Story 11 S11-R1 — §2/S7-R6 CLOSE the financial-column list and its order; Location is an identifier column not a financial one [S4-R12; S20-R19] so it never enters this list)</t>
         </is>
       </c>
       <c r="I44" s="2" t="inlineStr"/>
@@ -2923,7 +2923,7 @@
       </c>
       <c r="H51" s="2" t="inlineStr">
         <is>
-          <t>SV-8611 (SBC spec v12 2026-07-29 Story 13 S13-R1; S13-R2; S13-R3; S13-R4; S13-R7 — S13-R4 CLOSES the nine-toggle list and its order; Location is automatic and never a toggle [S4-R12; S4-R13])</t>
+          <t>SV-8611 (SBC spec v13 2026-07-31 Story 13 S13-R1; S13-R2; S13-R3; S13-R4; S13-R7 — S13-R4 CLOSES the nine-toggle list and its order; Location is automatic and never a toggle [S4-R12; S4-R13])</t>
         </is>
       </c>
       <c r="I51" s="2" t="inlineStr"/>
@@ -3019,7 +3019,7 @@
       </c>
       <c r="H53" s="2" t="inlineStr">
         <is>
-          <t>SV-8612; SV-8613 (SBC spec v12 2026-07-29 S14-R1; S14-R2; S15-R1; S15-R2; S20-R16 — these CLOSE the four-item menu and its verbatim labels; menu reshaped + "Print" removed per Chris Ward 2026-07-29 [newest-wins])</t>
+          <t>SV-8612; SV-8613 (SBC spec v13 2026-07-31 S14-R1; S14-R2; S15-R1; S15-R2; S20-R16 — these CLOSE the four-item menu and its verbatim labels; menu reshaped + "Print" removed per Chris Ward 2026-07-29 [newest-wins])</t>
         </is>
       </c>
       <c r="I53" s="2" t="inlineStr"/>
@@ -3361,7 +3361,7 @@
       </c>
       <c r="H60" s="2" t="inlineStr">
         <is>
-          <t>SV-8613 (SBC spec v12 2026-07-29 Story 15 S15-R7; S15-R8; S15-R9; S15-R10; S15-R11; S15-R14 + Story 4 S4-R13 — PDF header block; S15-R14/S4-R13 = the "Locations:" line in every export [Chris Ward 2026-07-29; newest-wins])</t>
+          <t>SV-8613 (SBC spec v13 2026-07-31 Story 15 S15-R7; S15-R8; S15-R9; S15-R10; S15-R11; S15-R14 + Story 4 S4-R13 — PDF header block; S15-R14/S4-R13 = the "Locations:" line in every export [Chris Ward 2026-07-29; newest-wins])</t>
         </is>
       </c>
       <c r="I60" s="2" t="inlineStr"/>
@@ -3606,7 +3606,7 @@
       </c>
       <c r="H65" s="2" t="inlineStr">
         <is>
-          <t>SV-8612; SV-8613; SV-8603 (SBC spec v12 2026-07-29 S14-R1; S14-R2; S14-R4; S15-R1; S15-R2; S15-R4; S15-R5; S4-R13 — the four-item Summary/Expanded menu; the Summary column list; the automatic Location column in every export)</t>
+          <t>SV-8612; SV-8613; SV-8603 (SBC spec v13 2026-07-31 S14-R1; S14-R2; S14-R4; S15-R1; S15-R2; S15-R4; S15-R5; S4-R13 — the four-item Summary/Expanded menu; the Summary column list; the automatic Location column in every export)</t>
         </is>
       </c>
       <c r="I65" s="2" t="inlineStr"/>

</xml_diff>